<commit_message>
Finalize secondary review of detailed design templates and samples
</commit_message>
<xml_diff>
--- a/詳細設計/01A_画面詳細設計書テンプレート.xlsx
+++ b/詳細設計/01A_画面詳細設計書テンプレート.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_表紙" sheetId="1" r:id="R9a178fe833b64390"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_改訂履歴" sheetId="2" r:id="Rf427e4c352b145e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_画面概要" sheetId="3" r:id="Re72eba32dab0496c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_画面レイアウト" sheetId="4" r:id="Rea0569623c614619"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_画面項目" sheetId="5" r:id="R3b7e35a8359d49fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Component_State" sheetId="6" r:id="R1ff32ebe54e549d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Event処理" sheetId="7" r:id="Rd72f97e58c0241c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_API_Mapping" sheetId="8" r:id="R4270dc4ab88c4624"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Message_例外" sheetId="9" r:id="R1212ab568cd24be6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_単体テスト観点" sheetId="10" r:id="Rd9a5200bb0b6401a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_表紙" sheetId="1" r:id="R83e42513d26b43a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_改訂履歴" sheetId="2" r:id="Rc0dfaa28821f4452"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_画面概要" sheetId="3" r:id="R6527f6b2a7b940c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_画面レイアウト" sheetId="4" r:id="R0278e212854647bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_画面項目" sheetId="5" r:id="Rd70a8b87afb64a15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Component_State" sheetId="6" r:id="Rb1fc64cf062748dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Event処理" sheetId="7" r:id="R6f8c93cc9b0b4db5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_API_Mapping" sheetId="8" r:id="Rf16100a0699541c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Message_例外" sheetId="9" r:id="R5a9bc492d1f240cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_単体テスト観点" sheetId="10" r:id="R0912c51be9864f43"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,6 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
   <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
@@ -412,7 +415,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="147">
+  <x:cellXfs count="148">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -850,6 +853,9 @@
     <x:xf numFmtId="0" fontId="4" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1389,43 +1395,22 @@
       <x:c r="K21" s="2"/>
       <x:c r="L21" s="2"/>
     </x:row>
-    <x:row r="22" ht="66" customHeight="1">
+    <x:row r="22" ht="100" customHeight="1">
       <x:c r="A22" s="58" t="str">
-        <x:v>本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
-      </x:c>
-      <x:c r="B22" s="59" t="str">
-        <x:v>本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
-      </x:c>
-      <x:c r="C22" s="59" t="str">
-        <x:v>本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
-      </x:c>
-      <x:c r="D22" s="59" t="str">
-        <x:v>本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
-      </x:c>
-      <x:c r="E22" s="59" t="str">
-        <x:v>本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
-      </x:c>
-      <x:c r="F22" s="59" t="str">
-        <x:v>本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
-      </x:c>
-      <x:c r="G22" s="59" t="str">
-        <x:v>本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
-      </x:c>
-      <x:c r="H22" s="59" t="str">
-        <x:v>本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
-      </x:c>
-      <x:c r="I22" s="59" t="str">
-        <x:v>本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
-      </x:c>
-      <x:c r="J22" s="59" t="str">
-        <x:v>本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
-      </x:c>
-      <x:c r="K22" s="59" t="str">
-        <x:v>本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
-      </x:c>
-      <x:c r="L22" s="60" t="str">
-        <x:v>本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
-      </x:c>
+        <x:v>文書状態：Review済／承認待ち。二次Review日：2026-09-30。
+本ファイルを複製し、基本設計から当該画面に存在する内容だけを設計する。画面主種別と適用機能を基準に、不要なSection、Placeholder、空行、空Blockは削除する。N/Aや「－」を並べず、基本設計にない機能・ITEM・State・Event・API・Testを推測して追加しない。完成後はITEM・VAL・EVT・API・MSG・UTの参照整合、孤立設計、重複記載を確認し、承認版に未管理のTBDを残さない。</x:v>
+      </x:c>
+      <x:c r="B22" s="59"/>
+      <x:c r="C22" s="59"/>
+      <x:c r="D22" s="59"/>
+      <x:c r="E22" s="59"/>
+      <x:c r="F22" s="59"/>
+      <x:c r="G22" s="59"/>
+      <x:c r="H22" s="59"/>
+      <x:c r="I22" s="59"/>
+      <x:c r="J22" s="59"/>
+      <x:c r="K22" s="59"/>
+      <x:c r="L22" s="60"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="61"/>
@@ -3691,30 +3676,30 @@
       <x:c r="K10" s="2"/>
       <x:c r="L10" s="2"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="84" customHeight="1">
       <x:c r="A11" s="111" t="str">
-        <x:v>&lt;&lt;Ver.x.x&gt;&gt;</x:v>
-      </x:c>
-      <x:c r="B11" s="111" t="str">
-        <x:v>&lt;&lt;yyyy-mm-dd&gt;&gt;</x:v>
+        <x:v>Ver.2.2</x:v>
+      </x:c>
+      <x:c r="B11" s="147" t="n">
+        <x:v>46295</x:v>
       </x:c>
       <x:c r="C11" s="111" t="str">
-        <x:v>&lt;&lt;新規／改訂／削除&gt;&gt;</x:v>
+        <x:v>Review</x:v>
       </x:c>
       <x:c r="D11" s="111" t="str">
-        <x:v>&lt;&lt;改訂内容&gt;&gt;</x:v>
+        <x:v>二次Review完了。設計内容変更なし。Review済／承認待ちへ整理。</x:v>
       </x:c>
       <x:c r="E11" s="111" t="str">
-        <x:v>&lt;&lt;記入&gt;&gt;</x:v>
+        <x:v>－</x:v>
       </x:c>
       <x:c r="F11" s="111" t="str">
-        <x:v>&lt;&lt;記入&gt;&gt;</x:v>
+        <x:v>Review済</x:v>
       </x:c>
       <x:c r="G11" s="111" t="str">
-        <x:v>&lt;&lt;記入&gt;&gt;</x:v>
+        <x:v>－</x:v>
       </x:c>
       <x:c r="H11" s="111" t="str">
-        <x:v>&lt;&lt;状態&gt;&gt;</x:v>
+        <x:v>承認待ち</x:v>
       </x:c>
       <x:c r="I11" s="2"/>
       <x:c r="J11" s="2"/>

</xml_diff>